<commit_message>
#45 PCB Completed BOM and Deliverables generated
</commit_message>
<xml_diff>
--- a/Design Files/Smart-Power-Supply-v6.0.0/BOM/Client_BOM.xlsx
+++ b/Design Files/Smart-Power-Supply-v6.0.0/BOM/Client_BOM.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="72">
   <si>
     <t>#</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t xml:space="preserve"> Remarks</t>
+    <t>#Column Name Error:' Remarks</t>
   </si>
   <si>
     <t>Capacitor</t>
@@ -86,10 +86,10 @@
     <t>J1</t>
   </si>
   <si>
-    <t>CONN HEADER SMD R/A 7POS 1.25MM</t>
-  </si>
-  <si>
-    <t>SM07B-GHS-TB(LF)(SN)</t>
+    <t>CONN HEADER SMD R/A 8POS 1.25MM</t>
+  </si>
+  <si>
+    <t>SM08B-GHS-TB(LF)(SN)</t>
   </si>
   <si>
     <t>JST</t>
@@ -113,6 +113,90 @@
     <t>XFCN</t>
   </si>
   <si>
+    <t>MOSFETs</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>MOSFET P-CH 20V 6.9A 6TSOP</t>
+  </si>
+  <si>
+    <t>6-TSOP_</t>
+  </si>
+  <si>
+    <t>IRLTS2242TRPBF</t>
+  </si>
+  <si>
+    <t>Infineon</t>
+  </si>
+  <si>
+    <t>MOSFET</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>MOSFET N-CH 60V 320MA SOT23-3</t>
+  </si>
+  <si>
+    <t>SOT-23</t>
+  </si>
+  <si>
+    <t>2N7002KT1G</t>
+  </si>
+  <si>
+    <t>ON Semiconductor</t>
+  </si>
+  <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>RES 10K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>Res-0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-0710KL</t>
+  </si>
+  <si>
+    <t>Yageo</t>
+  </si>
+  <si>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>R2, R3, R4, R5, R6, R8</t>
+  </si>
+  <si>
+    <t>RES 100K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-07100KL</t>
+  </si>
+  <si>
+    <t>100K</t>
+  </si>
+  <si>
+    <t>Resistors</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>RES SMD 97.6KOHM 0.1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RT0402BRD0797K6L</t>
+  </si>
+  <si>
+    <t>97.6K</t>
+  </si>
+  <si>
     <t>Switch</t>
   </si>
   <si>
@@ -141,6 +225,24 @@
   </si>
   <si>
     <t>XINGLIGHT</t>
+  </si>
+  <si>
+    <t>Opam</t>
+  </si>
+  <si>
+    <t>U5</t>
+  </si>
+  <si>
+    <t>IC CMOS 1 CIRCUIT SOT23-5</t>
+  </si>
+  <si>
+    <t>SOT-23-5</t>
+  </si>
+  <si>
+    <t>TLV271IDBVR</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
   </si>
 </sst>
 </file>
@@ -1259,8 +1361,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="6"/>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
     <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
@@ -1287,7 +1389,7 @@
       <c r="J1" s="14"/>
       <c r="K1" s="14"/>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" ht="15.75" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1418,7 +1520,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" ht="36.75" spans="1:11">
+    <row r="6" spans="1:11">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
         <f>ROW(B6)-ROW($B$2)</f>
@@ -1437,50 +1539,242 @@
         <v>31</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H6" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="13" t="s">
         <v>32</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>31</v>
       </c>
       <c r="J6" s="12">
         <v>1</v>
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" ht="36.75" spans="1:11">
+    <row r="7" ht="15.75" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
         <f>ROW(B7)-ROW($B$2)</f>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J7" s="9">
+        <v>1</v>
+      </c>
+      <c r="K7" s="9"/>
+    </row>
+    <row r="8" ht="15.75" spans="1:11">
+      <c r="A8" s="2"/>
+      <c r="B8" s="7">
+        <f>ROW(B8)-ROW($B$2)</f>
+        <v>6</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="J8" s="12">
+        <v>1</v>
+      </c>
+      <c r="K8" s="12"/>
+    </row>
+    <row r="9" ht="15.75" spans="1:11">
+      <c r="A9" s="2"/>
+      <c r="B9" s="7">
+        <f>ROW(B9)-ROW($B$2)</f>
+        <v>7</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="J9" s="9">
+        <v>6</v>
+      </c>
+      <c r="K9" s="9"/>
+    </row>
+    <row r="10" ht="15.75" spans="1:11">
+      <c r="A10" s="2"/>
+      <c r="B10" s="7">
+        <f>ROW(B10)-ROW($B$2)</f>
+        <v>8</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I10" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="J10" s="12">
+        <v>1</v>
+      </c>
+      <c r="K10" s="12"/>
+    </row>
+    <row r="11" ht="36.75" spans="1:11">
+      <c r="A11" s="2"/>
+      <c r="B11" s="7">
+        <f>ROW(B11)-ROW($B$2)</f>
+        <v>9</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="J11" s="9">
+        <v>1</v>
+      </c>
+      <c r="K11" s="9"/>
+    </row>
+    <row r="12" ht="36.75" spans="1:11">
+      <c r="A12" s="2"/>
+      <c r="B12" s="7">
+        <f>ROW(B12)-ROW($B$2)</f>
+        <v>10</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="I12" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="J12" s="12">
         <v>4</v>
       </c>
-      <c r="K7" s="9"/>
+      <c r="K12" s="12"/>
+    </row>
+    <row r="13" ht="15.75" spans="1:11">
+      <c r="A13" s="2"/>
+      <c r="B13" s="7">
+        <f>ROW(B13)-ROW($B$2)</f>
+        <v>11</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="J13" s="9">
+        <v>1</v>
+      </c>
+      <c r="K13" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>